<commit_message>
Match Excel Roles and Reboot column headers
Read the server list using Roles (UAG/CS) and Reboot (12 / 12:10)
instead of Component and Time.

Co-authored-by: manivannana27 <manivannana27@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/vcenter/sample_servers.xlsx
+++ b/vcenter/sample_servers.xlsx
@@ -424,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Component</t>
+          <t>Roles</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>Reboot</t>
         </is>
       </c>
     </row>

</xml_diff>